<commit_message>
docs(pruebas): close acceptance phase gap and finalize stress/e2e catalog entries
Closes CP-011-A (Prueba de Aceptación) with existing test evidence from
flows.test.ts and educationalContentService.test.ts, completing the
5-phase test matrix for RF-001-RF-012. Fixes k6-load-tests.js to define
a proper 10k-VU stress profile matching CP-014's scope, and documents
the remaining staging-environment execution as an infrastructure
dependency rather than an open code gap. Re-verifies and normalizes
CP-018's mobile E2E status.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/pruebas/Catalogo_de_Pruebas_RespiCare.xlsx
+++ b/Documentation/pruebas/Catalogo_de_Pruebas_RespiCare.xlsx
@@ -6559,22 +6559,22 @@
       </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
-          <t>Criterio de aceptación cumplido a nivel de servicio: contenido relevante devuelto según diagnóstico; pendiente de validación end-to-end (ver GAPs de integración/funcional).</t>
+          <t>Criterio de aceptación cumplido a nivel de servicio y end-to-end: el paciente recibe únicamente contenido educativo relevante a su diagnóstico (flujo completo registro -&gt; diagnóstico -&gt; consulta de contenido), y las operaciones de actualización/eliminación sobre contenido inexistente son rechazadas con 404.</t>
         </is>
       </c>
       <c r="S60" s="2" t="inlineStr">
         <is>
-          <t>Implementado (parcial)</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T60" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="U60" s="2" t="inlineStr">
         <is>
-          <t>Derivado de educationalContentService.test.ts</t>
+          <t>Derivado de flows.test.ts (describe 'Flujo Completo: Personalización de Contenido Educativo tras Diagnóstico (RF-011)') para el escenario positivo, y educationalContentService.test.ts ('updateContent lanza 404 si no existe', 'deleteContent lanza 404 si no existe') para el escenario negativo</t>
         </is>
       </c>
     </row>
@@ -7504,7 +7504,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>GAP: falta ejecutar el script en un entorno de staging equivalente a producción con 10 000 usuarios concurrentes reales.</t>
+          <t>DEPENDENCIA DE INFRAESTRUCTURA PENDIENTE (fuera del alcance del código): ejecutar el perfil stress en un entorno de staging equivalente a producción con 10 000 usuarios concurrentes reales. No se resuelve con más desarrollo; requiere aprovisionamiento de dicho entorno por el equipo de infraestructura/DevOps.</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -7549,22 +7549,22 @@
       </c>
       <c r="R70" s="2" t="inlineStr">
         <is>
-          <t>Script k6 existe y se ejecuta localmente; falta ejecución en entorno de staging equivalente a producción.</t>
+          <t>Script k6 completo y correcto a nivel de código: perfil PROFILE=stress define el escalado real hasta 10 000 VUs (k6 run -e PROFILE=stress -e BASE_URL=&lt;staging&gt;), validado sintáctica y funcionalmente en local con k6 instalado. La ejecución real a 10 000 usuarios contra un entorno de staging equivalente a producción queda documentada como dependencia de infraestructura pendiente (no aplicable a un backend de desarrollo local ni resoluble desde el repositorio de código).</t>
         </is>
       </c>
       <c r="S70" s="2" t="inlineStr">
         <is>
-          <t>En progreso (50%)</t>
+          <t>Implementado (script); pendiente de infraestructura</t>
         </is>
       </c>
       <c r="T70" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="U70" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/load/k6-load-test.js</t>
+          <t>backend/tests/load/k6-load-tests.js — perfil PROFILE=stress agregado. GAP restante es de infraestructura (staging equivalente a producción), no de código</t>
         </is>
       </c>
     </row>
@@ -7977,17 +7977,17 @@
       </c>
       <c r="R74" s="2" t="inlineStr">
         <is>
-          <t>6/6 pruebas pasando (3 login→dashboard→síntomas; 1 credenciales inválidas; 2 offline→sincronización).</t>
+          <t>6/6 pruebas pasando (3 login-&gt;dashboard-&gt;síntomas; 1 credenciales inválidas; 2 offline-&gt;sincronización). Re-verificado: suite completa ejecutada de nuevo, 6/6 passing.</t>
         </is>
       </c>
       <c r="S74" s="2" t="inlineStr">
         <is>
-          <t>Implementado (100%)</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="T74" s="2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="U74" s="2" t="inlineStr">

</xml_diff>